<commit_message>
refactor: Remove synthetic AI summarization in Step 2, preserve exact original review words with teencode and noise filtering
</commit_message>
<xml_diff>
--- a/Cleaned_sample_reviews.xlsx
+++ b/Cleaned_sample_reviews.xlsx
@@ -447,7 +447,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>[2. SỬA TEENCODE &amp; LỖI - AI TÓM TẮT Ý CHÍNH]</t>
+          <t>[2. SỬA TEENCODE &amp; LỖI]</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -547,17 +547,17 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Khen ngợi: nhân viên nhiệt tình, hiếu khách, thân thiện và nhanh nhẹn.</t>
+          <t>đóng gói hàng cẩn thận người giao hàng thân thiện dễ thương cho shop 5 sao nhé</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Khen_ngợi nhân_viên nhiệt_tình hiếu_khách thân_thiện nhanh_nhẹn</t>
+          <t>đóng_gói hàng cẩn_thận người giao_hàng thân_thiện dễ_thương shop 5</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Khen_ngợi, nhân_viên, nhiệt_tình, hiếu_khách, thân_thiện, nhanh_nhẹn</t>
+          <t>đóng_gói, hàng, cẩn_thận, người, giao_hàng, thân_thiện, dễ_thương, shop, 5</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -592,22 +592,22 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>excellent sản phẩm chất lượng and very nhanh vận chuyển khuyên dùng</t>
+          <t>chất lượng sản phẩm tuyệt vời và vận chuyển rất nhanh gợi ý</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>excellent sản phẩm chất lượng and very nhanh vận chuyển khuyên dùng</t>
+          <t>chất lượng sản phẩm tuyệt vời và vận chuyển rất nhanh gợi ý</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>excellent sản_phẩm_chất_lượng and_very nhanh vận_chuyển khuyên dùng</t>
+          <t>chất_lượng sản_phẩm tuyệt_vời vận_chuyển nhanh gợi_ý</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>excellent, sản_phẩm_chất_lượng, and_very, nhanh, vận_chuyển, khuyên, dùng</t>
+          <t>chất_lượng, sản_phẩm, tuyệt_vời, vận_chuyển, nhanh, gợi_ý</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>97%</t>
         </is>
       </c>
     </row>
@@ -697,27 +697,27 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Góp ý/Phản ánh: chất lượng món ăn chưa đạt chuẩn.</t>
+          <t>vải mát mặc thoải mái nhưng giao màu hơi nhạt hơn trong hình quảng cáo một chút</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Góp_ý Phản_ánh chất_lượng món ăn chưa đạt chuẩn</t>
+          <t>vải mát mặc thoải_mái giao màu nhạt hình_quảng_cáo một_chút</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Góp_ý, Phản_ánh, chất_lượng, món, ăn, chưa, đạt, chuẩn</t>
+          <t>vải, mát, mặc, thoải_mái, giao, màu, nhạt, hình_quảng_cáo, một_chút</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Tích cực</t>
+          <t>Tiêu cực</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>87%</t>
         </is>
       </c>
     </row>
@@ -742,32 +742,32 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>the item was bị hư hại during vận chuyển xấu tệ đóng gói</t>
+          <t>mặt hàng đã bị hư hỏng trong quá trình vận chuyển bao bì xấu</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>the item was bị hư hại during vận chuyển xấu tệ đóng gói</t>
+          <t>mặt hàng đã bị hư hỏng trong quá trình vận chuyển bao bì xấu</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>the item was hư_hại during vận_chuyển xấu_tệ đóng_gói</t>
+          <t>mặt_hàng hư_hỏng quá_trình vận_chuyển bao_bì xấu</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>the, item, was, hư_hại, during, vận_chuyển, xấu_tệ, đóng_gói</t>
+          <t>mặt_hàng, hư_hỏng, quá_trình, vận_chuyển, bao_bì, xấu</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Trung tính</t>
+          <t>Tiêu cực</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>97%</t>
         </is>
       </c>
     </row>
@@ -864,11 +864,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>71.4%</t>
+          <t>57.1%</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -884,11 +884,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>42.9%</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -904,11 +904,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -956,7 +956,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>vận chuyển</t>
+          <t>shop</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -966,11 +966,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>shop</t>
+          <t>vận chuyển</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -996,7 +996,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>khen ngợi</t>
+          <t>đóng gói</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -1006,7 +1006,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>nhân viên</t>
+          <t>hàng</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -1016,7 +1016,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>nhiệt tình</t>
+          <t>cẩn thận</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1026,7 +1026,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>hiếu khách</t>
+          <t>người</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1036,7 +1036,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>thân thiện</t>
+          <t>giao hàng</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1046,7 +1046,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>nhanh nhẹn</t>
+          <t>thân thiện</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -1056,7 +1056,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>excellent</t>
+          <t>dễ thương</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1066,7 +1066,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>sản phẩm chất lượng</t>
+          <t>sản phẩm</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1076,7 +1076,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>and very</t>
+          <t>tuyệt vời</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1096,7 +1096,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>khuyên</t>
+          <t>gợi ý</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1106,7 +1106,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>dùng</t>
+          <t>hàng giả</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1116,7 +1116,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>hàng giả</t>
+          <t>nhái</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1126,7 +1126,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>nhái</t>
+          <t>đừng</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1136,7 +1136,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>đừng</t>
+          <t>mua</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1222,7 +1222,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Khen ngợi nhân viên</t>
+          <t>đóng gói hàng</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -1237,7 +1237,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>nhân viên nhiệt tình</t>
+          <t>hàng cẩn thận</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1252,7 +1252,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>nhiệt tình hiếu khách</t>
+          <t>cẩn thận người</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -1267,7 +1267,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>hiếu khách thân thiện</t>
+          <t>người giao hàng</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -1282,7 +1282,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>thân thiện nhanh nhẹn</t>
+          <t>giao hàng thân thiện</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1297,7 +1297,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>excellent sản phẩm chất lượng</t>
+          <t>thân thiện dễ thương</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1312,7 +1312,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>sản phẩm chất lượng and very</t>
+          <t>dễ thương shop</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1327,7 +1327,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>and very nhanh</t>
+          <t>shop 5</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -1342,7 +1342,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>nhanh vận chuyển</t>
+          <t>chất lượng sản phẩm</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1357,7 +1357,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>vận chuyển khuyên</t>
+          <t>sản phẩm tuyệt vời</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1372,7 +1372,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>khuyên dùng</t>
+          <t>tuyệt vời vận chuyển</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1387,7 +1387,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>hàng giả nhái</t>
+          <t>vận chuyển nhanh</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -1402,7 +1402,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>nhái chất lượng</t>
+          <t>nhanh gợi ý</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1417,7 +1417,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>chất lượng đừng</t>
+          <t>hàng giả nhái</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1432,7 +1432,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>đừng mua</t>
+          <t>nhái chất lượng</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1447,7 +1447,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>mua lừa đảo</t>
+          <t>chất lượng đừng</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1455,14 +1455,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Tiêu cực</t>
+          <t>Tích cực</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>lừa đảo đấy</t>
+          <t>đừng mua</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1470,7 +1470,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Tiêu cực</t>
+          <t>Tích cực</t>
         </is>
       </c>
     </row>

</xml_diff>